<commit_message>
Update Author_ToConfirm with close-read extraction flags: rec 66 (F1 HIGH: overall-incidence IRRs absent from main paper which reports proportion-diagnosed-<50 RR; check online supplement, drives SENS2), rec 234 (F2 subgroup image eTable), rec 203/2131 (F3/F4 inert overlaps); rec 324 removed (fixed)
</commit_message>
<xml_diff>
--- a/meta_agents/search_v2/outputs/Author_ToConfirm.xlsx
+++ b/meta_agents/search_v2/outputs/Author_ToConfirm.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ToConfirm" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ToConfirm'!$A$1:$D$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ToConfirm'!$A$1:$D$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,13 +450,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="66" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,149 +484,149 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>155</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>41055508</t>
+          <t>36862439</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Lobular breast cancer statistics, 2025 (2025)</t>
+          <t>State Variation in Racial and Ethnic Disparities in Incidence of Triple-Negative Breast Cancer among US Women (2023)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>A. INCLUDED-extracted, no main PDF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>286</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>42118535</t>
+          <t>33074325</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Stage IV Breast Cancer Incidence and Survival, 2010-202 (2026)</t>
+          <t>Variation in breast cancer subtype incidence and distribution by race/ethnicity in the United States from 2010 to 2015 (2020)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Did not report the outcome of interest</t>
+          <t>A. INCLUDED-extracted, no main PDF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>209</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>40553473</t>
+          <t>36530732</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Breast Cancer Incidence Trends in Older US Women by Race, Ethnicity, Geography, and Stage (2025)</t>
+          <t>Racial and regional disparities of triple negative breast cancer incidence rates in the United States: An analysis of 2011-2019 NPCR and SEER incidence data (2022)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>B. INCLUDED-eligible, no PDF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>419</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>24670926</t>
+          <t>21656753</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Invasive cancer incidence - United States, 2010. (2014)</t>
+          <t>Higher population-based incidence rates of triple-negative breast cancer among young African-American women (2011)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>B. INCLUDED-eligible, no PDF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>2137</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>39853979</t>
+          <t>35119703</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Incidence Rate Trends of Breast Cancer Overall and by Molecular Subtype by Race and Ethnicity and Age (2025)</t>
+          <t>Cancer disparities among non-Hispanic urban American Indian and Alaska Native populations in the United States, 1999-2017 (2022)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>B. INCLUDED-eligible, no PDF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>4027</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>34427920</t>
+          <t>26661680</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Age distributions of breast cancer diagnosis and mortality by race and ethnicity in US women (2021)</t>
+          <t>Cancer incidence among Asian American populations in the United States, 2009-2011 (2016)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>G. EXTRACTION(low, overlap): overall IRRs not in text</t>
+          <t>B. INCLUDED-eligible, no PDF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>39132985</t>
+          <t>40553473</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Breast, Colorectal, and Prostate Cancer Incidence among Filipino Americans by Generational Status in the Multiethnic Cohort Study (2024)</t>
+          <t>Breast Cancer Incidence Trends in Older US Women by Race, Ethnicity, Geography, and Stage (2025)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -638,17 +638,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>24676851</t>
+          <t>24670926</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Disparities of cancer incidence in Michigan's American Indians: Spotlight on breast cancer (2014)</t>
+          <t>Invasive cancer incidence - United States, 2010. (2014)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -660,17 +660,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>32778443</t>
+          <t>39853979</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Are There Regional Differences in Triple Negative Breast Cancer among Non-Hispanic Black Women? (2021)</t>
+          <t>Incidence Rate Trends of Breast Cancer Overall and by Molecular Subtype by Race and Ethnicity and Age (2025)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -682,17 +682,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>21473509</t>
+          <t>39132985</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Persistence in breast cancer disparities between African Americans and whites in Wisconsin (2011)</t>
+          <t>Breast, Colorectal, and Prostate Cancer Incidence among Filipino Americans by Generational Status in the Multiethnic Cohort Study (2024)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -704,66 +704,66 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>119</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>36862439</t>
+          <t>24676851</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>State Variation in Racial and Ethnic Disparities in Incidence of Triple-Negative Breast Cancer among US Women (2023)</t>
+          <t>Disparities of cancer incidence in Michigan's American Indians: Spotlight on breast cancer (2014)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>A. INCLUDED-extracted, no main PDF</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>142</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>36301149</t>
+          <t>32778443</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, part 1: National cancer statistics (2022)</t>
+          <t>Are There Regional Differences in Triple Negative Breast Cancer among Non-Hispanic Black Women? (2021)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>145</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>16258086</t>
+          <t>21473509</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Breast cancer trends among black and white women in the United States (2005)</t>
+          <t>Persistence in breast cancer disparities between African Americans and whites in Wisconsin (2011)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
@@ -792,39 +792,39 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>210</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>36530732</t>
+          <t>34861613</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Racial and regional disparities of triple negative breast cancer incidence rates in the United States: An analysis of 2011-2019 NPCR and SEER incidence data (2022)</t>
+          <t>Breast cancer incidence trends in Asian women aged 20 or older as compared to other ethnic women in the United States from 2000 to 2018 by time period, age and tumor stage (2022)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>B. INCLUDED-eligible, no PDF</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>226</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>34861613</t>
+          <t>35113296</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Breast cancer incidence trends in Asian women aged 20 or older as compared to other ethnic women in the United States from 2000 to 2018 by time period, age and tumor stage (2022)</t>
+          <t>Home mortgage discrimination and incidence of triple-negative and Luminal A breast cancer among non-Hispanic Black and non-Hispanic White females in California, 2006–2015 (2022)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -836,17 +836,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>246</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>35113296</t>
+          <t>20567897</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Home mortgage discrimination and incidence of triple-negative and Luminal A breast cancer among non-Hispanic Black and non-Hispanic White females in California, 2006–2015 (2022)</t>
+          <t>Does socioeconomic disparity in cancer incidence vary across racial/ethnic groups? (2010)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -858,61 +858,61 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>252</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>42377954</t>
+          <t>32212335</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Breast Cancer Incidence in Asian American, Native Hawaiian, and Pacific Islander Populations, 2000-2022 (2026)</t>
+          <t>Forty-year trends in menopausal hormone therapy use and breast cancer incidence  among postmenopausal black and white women (2020)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>F. EXTRACTION: AANHPI subgroup rates in image eTable (verify Table 2/eTable)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>259</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>32162336</t>
+          <t>21850396</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, part I: National cancer statistics (2020)</t>
+          <t>What can we learn from the age- and race/ethnicity- specific rates of inflammatory breast carcinoma? (2011)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>284</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>20567897</t>
+          <t>42065927</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Does socioeconomic disparity in cancer incidence vary across racial/ethnic groups? (2010)</t>
+          <t>Trends in Female Breast Cancer Incidence among Japanese, Korean, and US Populations: An Age-Period-Cohort Analysis (2026)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -924,39 +924,39 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>251</t>
+          <t>310</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>32671723</t>
+          <t>18162138</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Triple-negative breast cancer incidence in the United States: ecological correlations with area-level sociodemographics, healthcare, and health behaviors (2021)</t>
+          <t>Recent breast cancer trends among Asian/Pacific Islander, Hispanic, and African-American women in the US: Changes by tumor subtype (2007)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Did not report the outcome of interest</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>316</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>32212335</t>
+          <t>29509274</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Forty-year trends in menopausal hormone therapy use and breast cancer incidence  among postmenopausal black and white women (2020)</t>
+          <t>Early estimates of cancer incidence for 2015: Expanding to include estimates for white and black races (2018)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -968,39 +968,39 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>369</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>10761199</t>
+          <t>29445940</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Breast cancer patterns and lifetime risk of developing breast cancer among Puerto Rican females. (2000)</t>
+          <t>Differences in breast cancer incidence among young women aged 20–49 years by stage and tumor characteristics, age, race, and ethnicity, 2004–2013 (2018)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>377</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>21850396</t>
+          <t>27792934</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>What can we learn from the age- and race/ethnicity- specific rates of inflammatory breast carcinoma? (2011)</t>
+          <t>Racial/ethnicity disparities in invasive breast cancer among younger and older  women: An analysis using multiple measures of population health (2016)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1012,17 +1012,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>284</t>
+          <t>402</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>42065927</t>
+          <t>26741869</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Trends in Female Breast Cancer Incidence among Japanese, Korean, and US Populations: An Age-Period-Cohort Analysis (2026)</t>
+          <t>Disparities in Breast Cancer Incidence, Mortality, and Quality of Care among African American and European American Women in South Carolina (2016)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1034,39 +1034,39 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>286</t>
+          <t>426</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>33074325</t>
+          <t>39837694</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Variation in breast cancer subtype incidence and distribution by race/ethnicity in the United States from 2010 to 2015 (2020)</t>
+          <t>Trends in Incidence of Invasive Lobular Carcinoma of the Breast by Race: Patterns by Age, Cancer Stage, and Socioeconomic Factors in the United States, 1992-2019 (2025)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>A. INCLUDED-extracted, no main PDF</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>474</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>18162138</t>
+          <t>41546752</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Recent breast cancer trends among Asian/Pacific Islander, Hispanic, and African-American women in the US: Changes by tumor subtype (2007)</t>
+          <t>Persistent poverty and breast cancer incidence by tumor subtype: intersections of rural/urban residence and race within USA Surveillance Epidemiology and End Results Registries, 2017 to 2021 (2026)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1078,17 +1078,17 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>477</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>29509274</t>
+          <t>41649619</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Early estimates of cancer incidence for 2015: Expanding to include estimates for white and black races (2018)</t>
+          <t>Spillover effects of public school integration in the southern United States: diverging trends in statewide annual breast cancer incidence, 2001–2019 (2026)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1100,83 +1100,83 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>504</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>27118258</t>
+          <t>40736150</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Risks of developing breast and colorectal cancer in association with incomes and geographic locations in Texas: A retrospective cohort study (2016)</t>
+          <t>Cancer Incidence and Trends in Persistent Poverty Areas of California by Race/Ethnicity and Sex (2025)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Did not report the outcome of interest</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>358</t>
+          <t>510</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>24343171</t>
+          <t>26766789</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the status of cancer, 1975-2010, featuring  prevalence of comorbidity and impact on survival among persons with lung, colorectal, breast, or prostate cancer (2014)</t>
+          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>362</t>
+          <t>516</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>28376154</t>
+          <t>37184135</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the Status of Cancer, 1975-2014, Featuring  Survival (2017)</t>
+          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>369</t>
+          <t>565</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>29445940</t>
+          <t>29120826</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Differences in breast cancer incidence among young women aged 20–49 years by stage and tumor characteristics, age, race, and ethnicity, 2004–2013 (2018)</t>
+          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1188,17 +1188,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>377</t>
+          <t>751</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>27792934</t>
+          <t>15090727</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Racial/ethnicity disparities in invasive breast cancer among younger and older  women: An analysis using multiple measures of population health (2016)</t>
+          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1210,39 +1210,39 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>754</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>16958083</t>
+          <t>38996557</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, 1975-2003, featuring cancer  among U.S. Hispanic/Latino populations (2006)</t>
+          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>998</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>26741869</t>
+          <t>28854891</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Disparities in Breast Cancer Incidence, Mortality, and Quality of Care among African American and European American Women in South Carolina (2016)</t>
+          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1254,105 +1254,101 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>25825511</t>
+          <t>37740603</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, 1975-2011, featuring incidence of breast cancer subtypes by race/ethnicity, poverty, and state (2015)</t>
+          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>415</t>
+          <t>1398</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>17929614</t>
+          <t>41989785</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Women's cancers among Alaska Natives 1969-2003. (2006)</t>
+          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>419</t>
+          <t>1453</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>21656753</t>
+          <t>41400551</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Higher population-based incidence rates of triple-negative breast cancer among young African-American women (2011)</t>
+          <t>American Cancer Society’s Report on the Status of Cancer Disparities in the United States, 2025 (2026)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>B. INCLUDED-eligible, no PDF</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>424</t>
+          <t>1457</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>12223421</t>
+          <t>41528114</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Breast cancer in a multiethnic cohort in Hawaii and Los Angeles: Risk factor-adjusted incidence in Japanese equals and in Hawaiians exceeds that in whites (2002)</t>
+          <t>Cancer statistics, 2026 (2026)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>426</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>39837694</t>
-        </is>
-      </c>
+          <t>1569</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Trends in Incidence of Invasive Lobular Carcinoma of the Breast by Race: Patterns by Age, Cancer Stage, and Socioeconomic Factors in the United States, 1992-2019 (2025)</t>
+          <t>Characterizing cancer patterns in Okinawan vs. mainland Japanese Americans: The Multiethnic Cohort Study (2025)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1364,39 +1360,39 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>1629</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>18323374</t>
+          <t>40189850</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Women's cancers among Alaska Natives: [corrected] 1969-2003. (2007)</t>
+          <t>Inequalities in Fertility-Impacting Cancer Incidence Among Young Populations in the United States (2025)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>474</t>
+          <t>1637</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>41546752</t>
+          <t>39808161</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Persistent poverty and breast cancer incidence by tumor subtype: intersections of rural/urban residence and race within USA Surveillance Epidemiology and End Results Registries, 2017 to 2021 (2026)</t>
+          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -1408,39 +1404,39 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>476</t>
+          <t>1800</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>41665696</t>
+          <t>38801414</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Rural–urban disparities in breast cancer incidence among US women aged 20–49: trends by race/ethnicity, stage, poverty, and state from 2000–2019 (2026)</t>
+          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>477</t>
+          <t>2440</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>41649619</t>
+          <t>31428891</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Spillover effects of public school integration in the southern United States: diverging trends in statewide annual breast cancer incidence, 2001–2019 (2026)</t>
+          <t>Cancer incidence and associations with known risk and protective factors: the Alaska EARTH study (2019)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1452,17 +1448,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>504</t>
+          <t>2453</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>40736150</t>
+          <t>31392297</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Cancer Incidence and Trends in Persistent Poverty Areas of California by Race/Ethnicity and Sex (2025)</t>
+          <t>Incidence and survival among young women with stage I-III breast cancer: Seer 2000-2015 (2019)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1474,17 +1470,13 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>510</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>26766789</t>
-        </is>
-      </c>
+          <t>3845</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Cancer statistics for Asian Americans, Native Hawaiians, and Pacific Islanders, 2016: Converging incidence in males and females (2016)</t>
+          <t>Characterizing inflammatory breast cancer among Arab Americans in the California, Detroit and New Jersey Surveillance, Epidemiology and End Results (SEER) registries (1988-2008) (2013)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1496,17 +1488,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>4043</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>37184135</t>
+          <t>37223193</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>The role of area-level socioeconomic disadvantage in racial disparities in cancer incidence in metropolitan Detroit (2023)</t>
+          <t>Trends in Breast Cancer Incidence and Mortality in the United States From 2004-2018: A Surveillance, Epidemiology, and End Results (SEER)-Based Study (2023)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1518,17 +1510,17 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>565</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>29120826</t>
+          <t>40257373</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Cancer in Guam and Hawaii: A comparison of two U.S. Island populations (2017)</t>
+          <t>Annual Report to the Nation on the Status of Cancer, featuring state-level statistics after the onset of the COVID-19 pandemic (2025)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1540,17 +1532,17 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>4294</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>15090727</t>
+          <t>39976243</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Population-based statistics for women diagnosed with inflammatory breast cancer (United States) (2004)</t>
+          <t>Cancer statistics for African American and Black people, 2025 (2025)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -1562,17 +1554,17 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>4389</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>38996557</t>
+          <t>24013772</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Breast cancer incidence and stage at diagnosis in the six US-Affiliated Pacific  Islands (2024)</t>
+          <t>Differences in the cancer burden among foreign-born and US-born Arab Americans living in metropolitan Detroit (2013)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1584,357 +1576,361 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>788</t>
+          <t>4429</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>31145458</t>
+          <t>28801942</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the Status of Cancer, Featuring Cancer in Men and Women Age 20–49 Years (2019)</t>
+          <t>Cancer risk in different generations of Middle Eastern immigrants to California, 1988-2013 (2017)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>C. INCLUDED-narrative, no PDF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>968</t>
+          <t>157</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>19998273</t>
+          <t>16258086</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, 1975-2006, featuring  colorectal cancer trends and impact of interventions (risk factors, screening, and treatment) to reduce future rates (2010)</t>
+          <t>Breast cancer trends among black and white women in the United States (2005)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>998</t>
+          <t>253</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>28854891</t>
+          <t>10761199</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Cancer-related risk factors and incidence of major cancers by race, gender and region; analysis of the NIH-AARP diet and health study (2017)</t>
+          <t>Breast cancer patterns and lifetime risk of developing breast cancer among Puerto Rican females. (2000)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>415</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>37740603</t>
+          <t>17929614</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Cancer incidence in the Somali population of Olmsted County: A Rochester epidemiology project study (2023)</t>
+          <t>Women's cancers among Alaska Natives 1969-2003. (2006)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>1398</t>
+          <t>424</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>41989785</t>
+          <t>12223421</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Early-Onset Cancer Incidence Disparities Between Black and White Individuals in the US, 2003-2022 (2026)</t>
+          <t>Breast cancer in a multiethnic cohort in Hawaii and Los Angeles: Risk factor-adjusted incidence in Japanese equals and in Hawaiians exceeds that in whites (2002)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>1453</t>
+          <t>428</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>41400551</t>
+          <t>18323374</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>American Cancer Society’s Report on the Status of Cancer Disparities in the United States, 2025 (2026)</t>
+          <t>Women's cancers among Alaska Natives: [corrected] 1969-2003. (2007)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>1457</t>
+          <t>476</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>41528114</t>
+          <t>41665696</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Cancer statistics, 2026 (2026)</t>
+          <t>Rural–urban disparities in breast cancer incidence among US women aged 20–49: trends by race/ethnicity, stage, poverty, and state from 2000–2019 (2026)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>1462</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>41742962</t>
-        </is>
-      </c>
+          <t>2038</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr"/>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Rising Breast Cancer Incidence and Poor Outcomes in Young Women: A Retrospective Study (2026)</t>
+          <t>Incidence trends in triple-negative breast cancer among women in the United States from 2010 to 2019 by race/ethnicity, age and tumor stage (2023)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Ineligible population</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>1569</t>
+          <t>3116</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Characterizing cancer patterns in Okinawan vs. mainland Japanese Americans: The Multiethnic Cohort Study (2025)</t>
+          <t>Time trends and racial differences in female breast cancer incidence in Pennsylvania, 1985-2004 (2011)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>1629</t>
+          <t>3268</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>40189850</t>
+          <t>17844709</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Inequalities in Fertility-Impacting Cancer Incidence Among Young Populations in the United States (2025)</t>
+          <t>Improving cancer incidence estimates for American Indians in Wisconsin (2007)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>1637</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>39808161</t>
+          <t>41055508</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Cancer Incidence in the Hispanic Community Health Study/Study of Latinos (HCHS/SOL)—The Onco-SOL Ancillary Study (2025)</t>
+          <t>Lobular breast cancer statistics, 2025 (2025)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>1800</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>38801414</t>
+          <t>42118535</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Rural–Urban Cancer Incidence and Trends in the United States, 2000 to 2019 (2024)</t>
+          <t>Stage IV Breast Cancer Incidence and Survival, 2010-202 (2026)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Did not report the outcome of interest</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2038</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr"/>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>36301149</t>
+        </is>
+      </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Incidence trends in triple-negative breast cancer among women in the United States from 2010 to 2019 by race/ethnicity, age and tumor stage (2023)</t>
+          <t>Annual report to the nation on the status of cancer, part 1: National cancer statistics (2022)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2131</t>
+          <t>235</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>35699957</t>
+          <t>32162336</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Associations of Obesity, Physical Activity, and Screening With State-Level Trends and Racial and Ethnic Disparities of Breast Cancer Incidence and Mortality in the US (2022)</t>
+          <t>Annual report to the nation on the status of cancer, part I: National cancer statistics (2020)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>G. EXTRACTION(low, overlap): subgroup rates in table</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2137</t>
+          <t>251</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>35119703</t>
+          <t>32671723</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Cancer disparities among non-Hispanic urban American Indian and Alaska Native populations in the United States, 1999-2017 (2022)</t>
+          <t>Triple-negative breast cancer incidence in the United States: ecological correlations with area-level sociodemographics, healthcare, and health behaviors (2021)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>B. INCLUDED-eligible, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Did not report the outcome of interest</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2151</t>
+          <t>321</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>34878180</t>
+          <t>27118258</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>American Cancer Society's report on the status of cancer disparities in the United States, 2021 (2022)</t>
+          <t>Risks of developing breast and colorectal cancer in association with incomes and geographic locations in Texas: A retrospective cohort study (2016)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>E. EXCLUDED w/o full text: Did not report the outcome of interest</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2163</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr"/>
+          <t>358</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>24343171</t>
+        </is>
+      </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
+          <t>Annual Report to the Nation on the status of cancer, 1975-2010, featuring  prevalence of comorbidity and impact on survival among persons with lung, colorectal, breast, or prostate cancer (2014)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -1946,101 +1942,105 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2440</t>
+          <t>362</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>31428891</t>
+          <t>28376154</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Cancer incidence and associations with known risk and protective factors: the Alaska EARTH study (2019)</t>
+          <t>Annual Report to the Nation on the Status of Cancer, 1975-2014, Featuring  Survival (2017)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2453</t>
+          <t>384</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>31392297</t>
+          <t>16958083</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Incidence and survival among young women with stage I-III breast cancer: Seer 2000-2015 (2019)</t>
+          <t>Annual report to the nation on the status of cancer, 1975-2003, featuring cancer  among U.S. Hispanic/Latino populations (2006)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>3116</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr"/>
+          <t>411</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>25825511</t>
+        </is>
+      </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Time trends and racial differences in female breast cancer incidence in Pennsylvania, 1985-2004 (2011)</t>
+          <t>Annual report to the nation on the status of cancer, 1975-2011, featuring incidence of breast cancer subtypes by race/ethnicity, poverty, and state (2015)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>3268</t>
+          <t>788</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>17844709</t>
+          <t>31145458</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Improving cancer incidence estimates for American Indians in Wisconsin (2007)</t>
+          <t>Annual Report to the Nation on the Status of Cancer, Featuring Cancer in Men and Women Age 20–49 Years (2019)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>D. EXCLUDED, not retrieved (POSSIBLE MISS)</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>3373</t>
+          <t>968</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>14974761</t>
+          <t>19998273</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Cancer Statistics, 2004 (2004)</t>
+          <t>Annual report to the nation on the status of cancer, 1975-2006, featuring  colorectal cancer trends and impact of interventions (risk factors, screening, and treatment) to reduce future rates (2010)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -2052,35 +2052,39 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>3429</t>
+          <t>1462</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>11814064</t>
+          <t>41742962</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Cancer statistics, 2002 (2002)</t>
+          <t>Rising Breast Cancer Incidence and Poor Outcomes in Young Women: A Retrospective Study (2026)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>E. EXCLUDED w/o full text: Ineligible population</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>3522</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr"/>
+          <t>2151</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>34878180</t>
+        </is>
+      </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the Status of Cancer, part 2: Early assessment of the COVID-19 pandemic’s impact on cancer diagnosis (2024)</t>
+          <t>American Cancer Society's report on the status of cancer disparities in the United States, 2021 (2022)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -2092,13 +2096,13 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>3713</t>
+          <t>2163</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
+          <t>Estrogen receptor negative breast cancer incidence rates are similar in Ghanaian and Non-Hispanic Black women in the USA (2022)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -2110,57 +2114,57 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>3845</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr"/>
+          <t>3373</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>14974761</t>
+        </is>
+      </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Characterizing inflammatory breast cancer among Arab Americans in the California, Detroit and New Jersey Surveillance, Epidemiology and End Results (SEER) registries (1988-2008) (2013)</t>
+          <t>Cancer Statistics, 2004 (2004)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>4027</t>
+          <t>3429</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>26661680</t>
+          <t>11814064</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Cancer incidence among Asian American populations in the United States, 2009-2011 (2016)</t>
+          <t>Cancer statistics, 2002 (2002)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>B. INCLUDED-eligible, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>4035</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>15221985</t>
-        </is>
-      </c>
+          <t>3522</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr"/>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, 1975-2001, with a special feature regarding survival (2004)</t>
+          <t>Annual Report to the Nation on the Status of Cancer, part 2: Early assessment of the COVID-19 pandemic’s impact on cancer diagnosis (2024)</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -2172,39 +2176,35 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>4043</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>37223193</t>
-        </is>
-      </c>
+          <t>3713</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Trends in Breast Cancer Incidence and Mortality in the United States From 2004-2018: A Surveillance, Epidemiology, and End Results (SEER)-Based Study (2023)</t>
+          <t>Cancer incidence and mortality among Filipinos in the USA and the Philippines: Patterns and trends (2016)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>4050</t>
+          <t>4035</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>23297039</t>
+          <t>15221985</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the Status of Cancer, 19752009, Featuring the Burden and Trends in Human Papillomavirus (HPV)Associated Cancers and HPV Vaccination Coverage Levels (2013)</t>
+          <t>Annual report to the nation on the status of cancer, 1975-2001, with a special feature regarding survival (2004)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -2216,17 +2216,17 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>4057</t>
+          <t>4050</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>21969133</t>
+          <t>23297039</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Breast cancer statistics, 2011 (2011)</t>
+          <t>Annual Report to the Nation on the Status of Cancer, 19752009, Featuring the Burden and Trends in Human Papillomavirus (HPV)Associated Cancers and HPV Vaccination Coverage Levels (2013)</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -2238,17 +2238,17 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>4065</t>
+          <t>4057</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>24399786</t>
+          <t>21969133</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Cancer Statistics, 2014 (2014)</t>
+          <t>Breast cancer statistics, 2011 (2011)</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -2260,17 +2260,17 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>4066</t>
+          <t>4065</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>21454908</t>
+          <t>24399786</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the Status of Cancer, 1975-2007, Featuring Tumors of the Brain and Other Nervous System (2011)</t>
+          <t>Cancer Statistics, 2014 (2014)</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -2282,17 +2282,17 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>4071</t>
+          <t>4066</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>12953083</t>
+          <t>21454908</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Annual report to the nation on the status of cancer, 1975-2000, featuring the uses of surveillance data for cancer prevention and control (2003)</t>
+          <t>Annual Report to the Nation on the Status of Cancer, 1975-2007, Featuring Tumors of the Brain and Other Nervous System (2011)</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -2304,22 +2304,22 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4071</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>40257373</t>
+          <t>12953083</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Annual Report to the Nation on the Status of Cancer, featuring state-level statistics after the onset of the COVID-19 pandemic (2025)</t>
+          <t>Annual report to the nation on the status of cancer, 1975-2000, featuring the uses of surveillance data for cancer prevention and control (2003)</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
@@ -2414,93 +2414,115 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>4294</t>
+          <t>4357</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>39976243</t>
+          <t>12924775</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Cancer statistics for African American and Black people, 2025 (2025)</t>
+          <t>Cancer statistics for Hispanics, 2003 (2003)</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>4357</t>
+          <t>66</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>12924775</t>
+          <t>34427920</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Cancer statistics for Hispanics, 2003 (2003)</t>
+          <t>Age distributions of breast cancer diagnosis and mortality by race and ethnicity in US women (2021)</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>E. EXCLUDED w/o full text: Overlapping or duplicate dataset</t>
+          <t>F1. EXTRACTION HIGH: overall-incidence IRRs NOT in main paper (paper reports proportion-diagnosed-&lt;50 RR, e.g. Hispanic 1.93). CHECK ONLINE SUPPLEMENT; drives SENS2. Likely reclassify to narrative.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>4389</t>
+          <t>234</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>24013772</t>
+          <t>42377954</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Differences in the cancer burden among foreign-born and US-born Arab Americans living in metropolitan Detroit (2013)</t>
+          <t>Breast Cancer Incidence in Asian American, Native Hawaiian, and Pacific Islander Populations, 2000-2022 (2026)</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>F2. EXTRACTION: AANHPI subgroup rates in image eTable (aggregates+NHW 139.5 already verified via supplement; verify 8 subgroup rates)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>4429</t>
+          <t>203</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>28801942</t>
+          <t>19001605</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Cancer risk in different generations of Middle Eastern immigrants to California, 1988-2013 (2017)</t>
+          <t>Recent trends in breast cancer among younger women in the United States (2008)</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>C. INCLUDED-narrative, no PDF</t>
+          <t>F3. EXTRACTION LOW (inert overlap): Black age-label &lt;30 vs &lt;40 mismatch; not selected anywhere</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2131</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>35699957</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Associations of Obesity, Physical Activity, and Screening With State-Level Trends and Racial and Ethnic Disparities of Breast Cancer Incidence and Mortality in the US (2022)</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>F4. EXTRACTION LOW (overlap): NHW 131.0 verified; subgroup rates in table</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D94"/>
+  <autoFilter ref="A1:D95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>